<commit_message>
1393A_313480kadar.pdf proformalarini listeye ekle
1393A_313480kadar.pdf icindeki 14 ayri proformadan (Elpim Muhendislik x2,
Depar Mekanik VRV klima, Metrans pompa, Krohne, Kanca Crane x4 vinc, Entek
Teknik PLC panosu, ETA Birkablo, Promek deprem kompansatoru x2, Radsan
topraklama) toplam 64 yeni kalem cikarilarak mevcut listeye eklendi. Liste
artik 81 proforma / 1096 kalem iceriyor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KcsznZgePm4VouW6FRZtG
</commit_message>
<xml_diff>
--- a/PROFORMA_FIYAT_LISTESI.xlsx
+++ b/PROFORMA_FIYAT_LISTESI.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Kalem Detay" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$68</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1033</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1097</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3255,8 +3255,620 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="n"/>
+      <c r="H69" t="n">
+        <v>9</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Kaynak metinde miktar sutunu bos birakilmis (qty=1 varsayildi) ve TOPLAM EURO satiri (line 88) rakam icermiyor - grand total belirtilmemis.</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>DEPAR MEKANIK A.S.</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>DM24.10.027</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>45574</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>VRV Klima Sistemi - TPAO Idil Elektrik Binasi</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>83731.81</v>
+      </c>
+      <c r="H70" t="n">
+        <v>2</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>KDV Haric genel toplam. Teklif Icmali sayfasinda 'Montaj Dahil Toplam Fiyat' olarak da 83.731,81 EUR gosteriliyor.</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>METRANS Makina Endustrisi Urunleri San. ve Tic. A.S.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>EO2402-TPAO-IDILSITE-COIL</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>45344</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TPAO IDIL SITE Crude Oil Transfer Pumps</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="n"/>
+      <c r="H71" t="n">
+        <v>4</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Bu belge esasen teknik datasheet paketidir; pompalarin ana/baz birim fiyati metinde hic gecmiyor (muhtemelen ayri/dahil edilmemis bir ticari sayfada). Sadece 'Optional Features' (opsiyonel test/kontrol) kalemleri fiyatlandirilmis; genel toplam verilmemis. KULLANICI KONTROL ETMELI.</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H72" t="n">
+        <v>8</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>TOTAL (KDV haric) = 17.500,00 EUR; VAT %20 = 3.500,00 EUR; grand total 6. arg olarak KDV DAHIL 21.000,00 EUR kullanildi.</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>4200.5</v>
+      </c>
+      <c r="H73" t="n">
+        <v>14</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>KDV haric. Kalem toplamlari (4.200,50) basilmis TOPLAM ile birebir uyumlu.</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>KANCA CRANE Makina Celik Sanayi Ticaret Limited Sirketi</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>KCM 2024/24511</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>45568</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>10 Ton Gezer Koprulu Vinc Sistemi</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="H74" t="n">
+        <v>1</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>KDV %20 haric genel toplam. KDV dahil genel toplam 2.520.000 TL (KDV %20 = 420.000 TL) olarak ayrica belirtilmis. Diger alt kalemler (kumanda panosu, elektrik tesisati, kopru imalati vb.) fiyat formunda 0 TL gosterilmis - ana sistem fiyatina dahil kabul edildi.</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>KANCA CRANE Makina Celik Sanayi Ticaret Limited Sirketi</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>KCM 2024/24512</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>45568</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>30 Ton Gezer Koprulu Vinc Sistemi</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="n">
+        <v>3150000</v>
+      </c>
+      <c r="H75" t="n">
+        <v>1</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>KDV %20 haric genel toplam. KDV dahil genel toplam 3.780.000 TL (KDV %20 = 630.000 TL) olarak ayrica belirtilmis. Diger alt kalemler 0 TL gosterilmis.</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>KANCA CRANE Makina Celik Sanayi Ticaret Limited Sirketi</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>KCM 2024/24512</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>45568</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>5 Ton Tek Koprulu Gezer Koprulu Vinc Sistemi</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="n">
+        <v>1350000</v>
+      </c>
+      <c r="H76" t="n">
+        <v>1</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>KDV %20 haric genel toplam. KDV dahil genel toplam 1.620.000 TL (KDV %20 = 270.000 TL) olarak ayrica belirtilmis. Kaynak metinde 'Rerans No' bu teklif icin de KCM 2024/24512 olarak basilmis (30 Ton teklifiyle ayni referans no - kaynak dokumanda muhtemel tekrar/hata, kullanici kontrol etmeli). Diger alt kalemler 0 TL gosterilmis.</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>KANCA CRANE Makina Celik Sanayi Ticaret Limited Sirketi</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>KCM 2024/24512</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>45568</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2 Ton Tek Koprulu Gezer Koprulu Vinc Sistemi</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="n">
+        <v>985000</v>
+      </c>
+      <c r="H77" t="n">
+        <v>1</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>KDV %20 haric genel toplam. KDV dahil genel toplam 1.182.000 TL (KDV %20 = 197.000 TL) olarak ayrica belirtilmis. Kaynak metinde 'Rerans No' bu teklif icin de KCM 2024/24512 (once gecen 30 Ton teklifiyle ayni referans no - kaynak dokumanda muhtemel tekrar/hata). Ayrica teknik ozellikler bolumunde 'Kaldirma Kapasitesi (Q): 30 TON' yazili (kopyala-yapistir hatasi olabilir) ama fiyat formu ve konu basligi acikca '2 TON' diyor - 2 Ton olarak kaydedildi. Diger alt kalemler 0 TL gosterilmis.</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Entek Teknik Malzeme Enerji Temsilcilik Tic. ve San. A.S.</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>45469</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Idil Pompaj Istasyonu PLC Paneli Temini ve Devreye Alinmasi</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="n">
+        <v>600000</v>
+      </c>
+      <c r="H78" t="n">
+        <v>1</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Alt Toplam (KDV haric) 500.000 EUR + KDV %20 (100.000 EUR) = Toplam (KDV dahil) 600.000 EUR; grand total 6. arg olarak KDV DAHIL rakam kullanildi.</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="n">
+        <v>3843802.84</v>
+      </c>
+      <c r="H79" t="n">
+        <v>12</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>TOPLAM (KDV haric) 3.203.169,03 TL + KDV %20 (640.633,81 TL) = GENEL TOPLAM (KDV dahil) 3.843.802,84 TL; grand total 6. arg olarak KDV DAHIL rakam kullanildi. Kaynak metinde ayrica sifir miktarli/fiyatli bir 'enstruman kablo notu' satiri (13 no) vardi, fiyatlandirilmis kalem olmadigi icin atlandi.</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>PROMEK Egitim ve Danismanlik Endustri Malzemeleri Insaat Taahhut Ithalat Ihracat Sanayi Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>TUM24/002</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>45570</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Kardan Mafsalli Deprem Kompansatoru Teklifi</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="n">
+        <v>343005.6</v>
+      </c>
+      <c r="H80" t="n">
+        <v>2</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Fiyatlara KDV dahil degildir (KDV haric).</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>RADSAN</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>KR2400000000592</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Topraklama Malzemeleri Teklifi</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="n">
+        <v>40051</v>
+      </c>
+      <c r="H81" t="n">
+        <v>7</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Fiyatlara %20 KDV dahil degildir (KDV haric).</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>PROMEK Egitim ve Danismanlik Endustri Malzemeleri Insaat Taahhut Ithalat Ihracat Sanayi Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>TUM24/003</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>45582</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Kardan Mafsalli Deprem Kompansatoru Teklifi</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="n">
+        <v>103860</v>
+      </c>
+      <c r="H82" t="n">
+        <v>1</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Fiyatlara KDV dahil degildir (KDV haric).</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J68"/>
+  <autoFilter ref="A1:J82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3267,7 +3879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1033"/>
+  <dimension ref="A1:L1097"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -56760,8 +57372,3336 @@
         </is>
       </c>
     </row>
+    <row r="1034">
+      <c r="A1034" t="n">
+        <v>1033</v>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1034" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>CORTEM EVL-070070 LED Yuksek Tavan Armaturu, 70W, 7.852 Lumen, Ex II 2G Ex db eb op is IIC T4/T5 Gb, IP66</t>
+        </is>
+      </c>
+      <c r="G1034" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1034" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1034" s="3" t="n">
+        <v>609.5</v>
+      </c>
+      <c r="J1034" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1034" s="3" t="n">
+        <v>609.5</v>
+      </c>
+      <c r="L1034" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="n">
+        <v>1034</v>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1035" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>CORTEM EVL-080100 LED Yuksek Tavan Armaturu, 130W, 12.653 Lumen, Ex II 2G Ex db eb op is IIC T4/T5 Gb, IP66</t>
+        </is>
+      </c>
+      <c r="G1035" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1035" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1035" s="3" t="n">
+        <v>825.5</v>
+      </c>
+      <c r="J1035" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1035" s="3" t="n">
+        <v>825.5</v>
+      </c>
+      <c r="L1035" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="n">
+        <v>1035</v>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1036" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>CORTEM CSC-216 Exproof Anahtar, 16A, 0-1 Acma/Kapama, EEx d IIC T6, IP66, 2x1" kablo girisli</t>
+        </is>
+      </c>
+      <c r="G1036" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1036" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1036" s="3" t="n">
+        <v>117.4</v>
+      </c>
+      <c r="J1036" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1036" s="3" t="n">
+        <v>117.4</v>
+      </c>
+      <c r="L1036" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="n">
+        <v>1036</v>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1037" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>CORTEM SX-26.1 Exproof Buat, EEx d IIC T6, IP66, 4x3/4" kablo girisli</t>
+        </is>
+      </c>
+      <c r="G1037" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1037" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1037" s="3" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J1037" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1037" s="3" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="L1037" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="n">
+        <v>1037</v>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1038" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>CORTEM PY-216B + SPY-216B Exproof Priz-Fis Takimi, 16A, 2P+PE, 220V, EEx d IIC T6, IP66</t>
+        </is>
+      </c>
+      <c r="G1038" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1038" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1038" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="J1038" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1038" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="L1038" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="n">
+        <v>1038</v>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1039" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>CORTEM PY-432R + SPY-432R Exproof Priz-Fis Takimi, 16A, 3P+N+PE, 380V, EEx d IIC T6, IP66</t>
+        </is>
+      </c>
+      <c r="G1039" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1039" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1039" s="3" t="n">
+        <v>339.3</v>
+      </c>
+      <c r="J1039" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1039" s="3" t="n">
+        <v>339.3</v>
+      </c>
+      <c r="L1039" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="n">
+        <v>1039</v>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1040" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>Exproof Start/Stop pushbutonu (kontaklari dahil), 2x1" girisli</t>
+        </is>
+      </c>
+      <c r="G1040" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1040" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1040" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="J1040" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1040" s="3" t="n">
+        <v>141</v>
+      </c>
+      <c r="L1040" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="n">
+        <v>1040</v>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1041" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>CORTEM CSC-R Exproof Acil Stop Butonu, EEx d IIC T6, IP66, 2x1" girisli</t>
+        </is>
+      </c>
+      <c r="G1041" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1041" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1041" s="3" t="n">
+        <v>121.5</v>
+      </c>
+      <c r="J1041" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1041" s="3" t="n">
+        <v>121.5</v>
+      </c>
+      <c r="L1041" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="n">
+        <v>1041</v>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>TEKLIF TALEBI (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1042" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>(TPAO) Idil Sirnak Depolama Tesisi TEKLIF TALEBI</t>
+        </is>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>CORTEM SAG-302318 Ex Terminal Kutusu, montaj plakasi dahil, EEx d IIC T6, IP66, 305x230x190mm</t>
+        </is>
+      </c>
+      <c r="G1042" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1042" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1042" s="3" t="n">
+        <v>128</v>
+      </c>
+      <c r="J1042" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1042" s="3" t="n">
+        <v>128</v>
+      </c>
+      <c r="L1042" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="n">
+        <v>1042</v>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>DEPAR MEKANIK A.S.</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>DM24.10.027</t>
+        </is>
+      </c>
+      <c r="D1043" s="2" t="n">
+        <v>45574</v>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>VRV Klima Sistemi - TPAO Idil Elektrik Binasi</t>
+        </is>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>DAIKIN VRV IV Heat Pump C+ Cold Region VRV Klima Sistemi - cihaz paketi (dis uniteler RXYLQ10T/RXYLQ26T, ic uniteler FXZQ/FXFQ serisi, kumandalar, BS-unit vb, 15 kalem)</t>
+        </is>
+      </c>
+      <c r="G1043" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>Paket</t>
+        </is>
+      </c>
+      <c r="I1043" s="3" t="n">
+        <v>62023.56</v>
+      </c>
+      <c r="J1043" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1043" s="3" t="n">
+        <v>62023.56</v>
+      </c>
+      <c r="L1043" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="n">
+        <v>1043</v>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>DEPAR MEKANIK A.S.</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>DM24.10.027</t>
+        </is>
+      </c>
+      <c r="D1044" s="2" t="n">
+        <v>45574</v>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>VRV Klima Sistemi - TPAO Idil Elektrik Binasi</t>
+        </is>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>VRV Klima Sistemi Montaji (bakir boru/izolasyon/joint montaji, ic-dis unite baglantilari, kumanda montaji, azot testi, vakum, gaz sarji, devreye alma)</t>
+        </is>
+      </c>
+      <c r="G1044" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>Paket</t>
+        </is>
+      </c>
+      <c r="I1044" s="3" t="n">
+        <v>21708.25</v>
+      </c>
+      <c r="J1044" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1044" s="3" t="n">
+        <v>21708.25</v>
+      </c>
+      <c r="L1044" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="n">
+        <v>1044</v>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>METRANS Makina Endustrisi Urunleri San. ve Tic. A.S.</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>EO2402-TPAO-IDILSITE-COIL</t>
+        </is>
+      </c>
+      <c r="D1045" s="2" t="n">
+        <v>45344</v>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>TPAO IDIL SITE Crude Oil Transfer Pumps</t>
+        </is>
+      </c>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>Item 1 (340 m3/h - 355m, Model 3600 6x8-14AD, S-6) - Witness unit test with job motor/coupling/baseplate (APIHI-CUT1) opsiyonel ek</t>
+        </is>
+      </c>
+      <c r="G1045" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1045" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1045" s="3" t="n">
+        <v>4846.43</v>
+      </c>
+      <c r="J1045" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1045" s="3" t="n">
+        <v>14539.29</v>
+      </c>
+      <c r="L1045" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="n">
+        <v>1045</v>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>METRANS Makina Endustrisi Urunleri San. ve Tic. A.S.</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>EO2402-TPAO-IDILSITE-COIL</t>
+        </is>
+      </c>
+      <c r="D1046" s="2" t="n">
+        <v>45344</v>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>TPAO IDIL SITE Crude Oil Transfer Pumps</t>
+        </is>
+      </c>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>Item 1 (340 m3/h - 355m, Model 3600 6x8-14AD, S-6) - Witnessed mounting pad flatness check on baseplate per API opsiyonel ek</t>
+        </is>
+      </c>
+      <c r="G1046" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1046" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1046" s="3" t="n">
+        <v>608.35</v>
+      </c>
+      <c r="J1046" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1046" s="3" t="n">
+        <v>1825.05</v>
+      </c>
+      <c r="L1046" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="n">
+        <v>1046</v>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>METRANS Makina Endustrisi Urunleri San. ve Tic. A.S.</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>EO2402-TPAO-IDILSITE-COIL</t>
+        </is>
+      </c>
+      <c r="D1047" s="2" t="n">
+        <v>45344</v>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>TPAO IDIL SITE Crude Oil Transfer Pumps</t>
+        </is>
+      </c>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>Item 2 (165 m3/h - 355m, Model 3600 4x6-10, S-6) - Witnessed mounting pad flatness check on baseplate per API opsiyonel ek</t>
+        </is>
+      </c>
+      <c r="G1047" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1047" s="3" t="n">
+        <v>538.17</v>
+      </c>
+      <c r="J1047" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1047" s="3" t="n">
+        <v>1076.34</v>
+      </c>
+      <c r="L1047" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="n">
+        <v>1047</v>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>METRANS Makina Endustrisi Urunleri San. ve Tic. A.S.</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>EO2402-TPAO-IDILSITE-COIL</t>
+        </is>
+      </c>
+      <c r="D1048" s="2" t="n">
+        <v>45344</v>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>TPAO IDIL SITE Crude Oil Transfer Pumps</t>
+        </is>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>Item 2 (165 m3/h - 355m, Model 3600 4x6-10, S-6) - Witness unit test with job motor/coupling/baseplate (APIHI-CUT1) opsiyonel ek</t>
+        </is>
+      </c>
+      <c r="G1048" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1048" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1048" s="3" t="n">
+        <v>4846.43</v>
+      </c>
+      <c r="J1048" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1048" s="3" t="n">
+        <v>9692.860000000001</v>
+      </c>
+      <c r="L1048" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="n">
+        <v>1048</v>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1049" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F1049" t="inlineStr">
+        <is>
+          <t>Pressure Ind. Transmitter</t>
+        </is>
+      </c>
+      <c r="G1049" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1049" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1049" s="3" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J1049" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1049" s="3" t="n">
+        <v>3500</v>
+      </c>
+      <c r="L1049" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="n">
+        <v>1049</v>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1050" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>Pressure Indicator</t>
+        </is>
+      </c>
+      <c r="G1050" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1050" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1050" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="J1050" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1050" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="L1050" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="n">
+        <v>1050</v>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1051" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>Temperature Indicator</t>
+        </is>
+      </c>
+      <c r="G1051" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1051" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1051" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="J1051" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1051" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="L1051" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="n">
+        <v>1051</v>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1052" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>Level Switch</t>
+        </is>
+      </c>
+      <c r="G1052" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1052" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1052" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J1052" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1052" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="L1052" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="n">
+        <v>1052</v>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1053" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E1053" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F1053" t="inlineStr">
+        <is>
+          <t>Diff. Pressure Indicator</t>
+        </is>
+      </c>
+      <c r="G1053" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1053" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1053" s="3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J1053" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1053" s="3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L1053" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="n">
+        <v>1053</v>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1054" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E1054" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F1054" t="inlineStr">
+        <is>
+          <t>Temp. Ind. Transmitter</t>
+        </is>
+      </c>
+      <c r="G1054" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1054" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1054" s="3" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J1054" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1054" s="3" t="n">
+        <v>3500</v>
+      </c>
+      <c r="L1054" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="n">
+        <v>1054</v>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1055" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F1055" t="inlineStr">
+        <is>
+          <t>Flow Switch</t>
+        </is>
+      </c>
+      <c r="G1055" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1055" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1055" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J1055" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1055" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="L1055" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="n">
+        <v>1055</v>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>KROHNE Otomasyon Sanayi ve Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1056" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E1056" t="inlineStr">
+        <is>
+          <t>TUMAS Turk Muhendislik - Enstruman Proforma Faturasi</t>
+        </is>
+      </c>
+      <c r="F1056" t="inlineStr">
+        <is>
+          <t>Level Indicator</t>
+        </is>
+      </c>
+      <c r="G1056" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1056" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1056" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="J1056" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1056" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="L1056" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="n">
+        <v>1056</v>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1057" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1057" t="inlineStr">
+        <is>
+          <t>CORTEM FLOWEX-080070 LED Armatur, 70W, 9.547 lm, IP66, 5000K, Ex db eb mb IIC T5/86C, Zone 1/21</t>
+        </is>
+      </c>
+      <c r="G1057" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1057" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1057" s="3" t="n">
+        <v>609.7</v>
+      </c>
+      <c r="J1057" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1057" s="3" t="n">
+        <v>609.7</v>
+      </c>
+      <c r="L1057" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="n">
+        <v>1057</v>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1058" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1058" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1058" t="inlineStr">
+        <is>
+          <t>CORTEM CSCD-216 vaviyen 1-2 Anahtar, 16A, Ex db IIC T6, IP66, Zone 1/21</t>
+        </is>
+      </c>
+      <c r="G1058" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1058" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1058" s="3" t="n">
+        <v>117.4</v>
+      </c>
+      <c r="J1058" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1058" s="3" t="n">
+        <v>117.4</v>
+      </c>
+      <c r="L1058" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="n">
+        <v>1058</v>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1059" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1059" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1059" t="inlineStr">
+        <is>
+          <t>CORTEM LIFEX-ME-1230N Acil Aydinlatma Armaturu, Lineer LED 30W 4.112lm, Ni-Cd batarya 180dk, IP66, Zone1/21</t>
+        </is>
+      </c>
+      <c r="G1059" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1059" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1059" s="3" t="n">
+        <v>490.1</v>
+      </c>
+      <c r="J1059" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1059" s="3" t="n">
+        <v>490.1</v>
+      </c>
+      <c r="L1059" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="n">
+        <v>1059</v>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1060" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1060" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1060" t="inlineStr">
+        <is>
+          <t>CORTEM CSC-216 normal anahtar, 16A, Ex db IIC T6, IP66, Zone 1/21</t>
+        </is>
+      </c>
+      <c r="G1060" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1060" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1060" s="3" t="n">
+        <v>114.5</v>
+      </c>
+      <c r="J1060" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1060" s="3" t="n">
+        <v>114.5</v>
+      </c>
+      <c r="L1060" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="n">
+        <v>1060</v>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1061" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1061" t="inlineStr">
+        <is>
+          <t>CORTEM ST-26.1 buat, 3x3/4" girisli, Exd IIC Gb, IP66, Zone 1/21</t>
+        </is>
+      </c>
+      <c r="G1061" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1061" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1061" s="3" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J1061" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1061" s="3" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="L1061" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="n">
+        <v>1061</v>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1062" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1062" t="inlineStr">
+        <is>
+          <t>CORTEM SL-26.1 buat, 2x3/4" girisli, Exd IIC Gb, IP66, Zone 1/21</t>
+        </is>
+      </c>
+      <c r="G1062" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1062" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1062" s="3" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="J1062" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1062" s="3" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="L1062" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="n">
+        <v>1062</v>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1063" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1063" t="inlineStr">
+        <is>
+          <t>CORTEM ELF-2 3/4" dirsek, Ex db IIC Gb, IP66/67, Zone 1/2</t>
+        </is>
+      </c>
+      <c r="G1063" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1063" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1063" s="3" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="J1063" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1063" s="3" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="L1063" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="n">
+        <v>1063</v>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1064" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>CORTEM EYS-2 3/4" Durdurucu, Ex db IIC Gb, IP66/67, Zone 1/2</t>
+        </is>
+      </c>
+      <c r="G1064" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1064" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1064" s="3" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="J1064" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1064" s="3" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="L1064" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="n">
+        <v>1064</v>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1065" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>CORTEM EM-2 3/4" mansson, Ex db IIB Gb, IP66/67, Zone 1/2</t>
+        </is>
+      </c>
+      <c r="G1065" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1065" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1065" s="3" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="J1065" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1065" s="3" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="L1065" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="n">
+        <v>1065</v>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1066" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1066" t="inlineStr">
+        <is>
+          <t>CORTEM PY-216B 16A Monofaze priz ve fis, Ex d IIC T6 Gb, Zone 1/2</t>
+        </is>
+      </c>
+      <c r="G1066" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1066" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1066" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="J1066" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1066" s="3" t="n">
+        <v>216</v>
+      </c>
+      <c r="L1066" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="n">
+        <v>1066</v>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1067" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1067" t="inlineStr">
+        <is>
+          <t>CORTEM PY-432R 16A Trifaze priz ve fis, Ex d IIC T6 Gb, Zone 1/2</t>
+        </is>
+      </c>
+      <c r="G1067" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1067" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1067" s="3" t="n">
+        <v>339.3</v>
+      </c>
+      <c r="J1067" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1067" s="3" t="n">
+        <v>339.3</v>
+      </c>
+      <c r="L1067" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="n">
+        <v>1067</v>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1068" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1068" t="inlineStr">
+        <is>
+          <t>CORTEM BMF-2 3/4" uc parcali rekor erkek-disi, Ex db IIB Gb, IP66/67, Zone 1/2</t>
+        </is>
+      </c>
+      <c r="G1068" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1068" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1068" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1068" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1068" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L1068" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="n">
+        <v>1068</v>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1069" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1069" t="inlineStr">
+        <is>
+          <t>CORTEM LBHS-2 3/4" kapakli dirsek, Ex d IIB, IP66, Zone 1/21</t>
+        </is>
+      </c>
+      <c r="G1069" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1069" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1069" s="3" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="J1069" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1069" s="3" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="L1069" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="n">
+        <v>1069</v>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>ELPIM Muhendislik Musavirlik Elektrik San. ve Tic. Ltd. Sti</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>TEKLIF (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1070" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>TPAO Idil Sirnak Depolama Tesisi</t>
+        </is>
+      </c>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>FITRE TASS22 AD Telefon, Ex e mb (ib) IIC T5, IP66</t>
+        </is>
+      </c>
+      <c r="G1070" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1070" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1070" s="3" t="n">
+        <v>2198</v>
+      </c>
+      <c r="J1070" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1070" s="3" t="n">
+        <v>2198</v>
+      </c>
+      <c r="L1070" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="n">
+        <v>1070</v>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>KANCA CRANE Makina Celik Sanayi Ticaret Limited Sirketi</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>KCM 2024/24511</t>
+        </is>
+      </c>
+      <c r="D1071" s="2" t="n">
+        <v>45568</v>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>10 Ton Gezer Koprulu Vinc Sistemi</t>
+        </is>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>10 Ton cift kiris tipi gezer koprulu tavan vinc sistemi (kaldirma grubu, kumanda panosu, kopru basligi, elektrik tesisati dahil komple sistem)</t>
+        </is>
+      </c>
+      <c r="G1071" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1071" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1071" s="3" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="J1071" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1071" s="3" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="L1071" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="n">
+        <v>1071</v>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>KANCA CRANE Makina Celik Sanayi Ticaret Limited Sirketi</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>KCM 2024/24512</t>
+        </is>
+      </c>
+      <c r="D1072" s="2" t="n">
+        <v>45568</v>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>30 Ton Gezer Koprulu Vinc Sistemi</t>
+        </is>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>30 Ton cift kiris tipi gezer koprulu tavan vinc sistemi (kaldirma grubu, kumanda panosu, kopru basligi, elektrik tesisati dahil komple sistem)</t>
+        </is>
+      </c>
+      <c r="G1072" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1072" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1072" s="3" t="n">
+        <v>3150000</v>
+      </c>
+      <c r="J1072" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1072" s="3" t="n">
+        <v>3150000</v>
+      </c>
+      <c r="L1072" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="n">
+        <v>1072</v>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>KANCA CRANE Makina Celik Sanayi Ticaret Limited Sirketi</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>KCM 2024/24512</t>
+        </is>
+      </c>
+      <c r="D1073" s="2" t="n">
+        <v>45568</v>
+      </c>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>5 Ton Tek Koprulu Gezer Koprulu Vinc Sistemi</t>
+        </is>
+      </c>
+      <c r="F1073" t="inlineStr">
+        <is>
+          <t>5 Ton tek kiris tipi gezer koprulu tavan vinc sistemi (kaldirma grubu, kumanda panosu, kopru basligi, elektrik tesisati dahil komple sistem)</t>
+        </is>
+      </c>
+      <c r="G1073" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1073" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1073" s="3" t="n">
+        <v>1350000</v>
+      </c>
+      <c r="J1073" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1073" s="3" t="n">
+        <v>1350000</v>
+      </c>
+      <c r="L1073" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="n">
+        <v>1073</v>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>KANCA CRANE Makina Celik Sanayi Ticaret Limited Sirketi</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>KCM 2024/24512</t>
+        </is>
+      </c>
+      <c r="D1074" s="2" t="n">
+        <v>45568</v>
+      </c>
+      <c r="E1074" t="inlineStr">
+        <is>
+          <t>2 Ton Tek Koprulu Gezer Koprulu Vinc Sistemi</t>
+        </is>
+      </c>
+      <c r="F1074" t="inlineStr">
+        <is>
+          <t>2 Ton tek kiris tipi gezer koprulu tavan vinc sistemi (kaldirma grubu, kumanda panosu, kopru basligi, elektrik tesisati dahil komple sistem)</t>
+        </is>
+      </c>
+      <c r="G1074" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1074" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1074" s="3" t="n">
+        <v>985000</v>
+      </c>
+      <c r="J1074" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1074" s="3" t="n">
+        <v>985000</v>
+      </c>
+      <c r="L1074" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="n">
+        <v>1074</v>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Entek Teknik Malzeme Enerji Temsilcilik Tic. ve San. A.S.</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>PROFORMA FATURA (Ref yok)</t>
+        </is>
+      </c>
+      <c r="D1075" s="2" t="n">
+        <v>45469</v>
+      </c>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>Idil Pompaj Istasyonu PLC Paneli Temini ve Devreye Alinmasi</t>
+        </is>
+      </c>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>Idil Pompaj Istasyonu PLC Paneli Temini ve Devreye Alinmasi (10 adet Pompa PLC Sistemi, CPU, haberlesme/network kartlari, 10" HMI, IS bariyerleri, pano ici baglantilar, yazilim ve lisanslar dahil)</t>
+        </is>
+      </c>
+      <c r="G1075" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1075" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1075" s="3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J1075" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1075" s="3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="L1075" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="n">
+        <v>1075</v>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1076" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1076" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl BLACK 1x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1076" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1076" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1076" s="3" t="n">
+        <v>49.4349</v>
+      </c>
+      <c r="J1076" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1076" s="3" t="n">
+        <v>49434.9</v>
+      </c>
+      <c r="L1076" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="n">
+        <v>1076</v>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1077" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1077" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 2x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1077" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1077" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1077" s="3" t="n">
+        <v>93.54519999999999</v>
+      </c>
+      <c r="J1077" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1077" s="3" t="n">
+        <v>93545.2</v>
+      </c>
+      <c r="L1077" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="n">
+        <v>1077</v>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1078" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1078" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 4x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1078" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1078" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1078" s="3" t="n">
+        <v>138.9711</v>
+      </c>
+      <c r="J1078" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1078" s="3" t="n">
+        <v>138971.1</v>
+      </c>
+      <c r="L1078" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="n">
+        <v>1078</v>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1079" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1079" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 6x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1079" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1079" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1079" s="3" t="n">
+        <v>212.1013</v>
+      </c>
+      <c r="J1079" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1079" s="3" t="n">
+        <v>212101.3</v>
+      </c>
+      <c r="L1079" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="n">
+        <v>1079</v>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1080" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 8x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1080" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1080" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1080" s="3" t="n">
+        <v>255.2821</v>
+      </c>
+      <c r="J1080" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1080" s="3" t="n">
+        <v>255282.1</v>
+      </c>
+      <c r="L1080" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="n">
+        <v>1080</v>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1081" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 10x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1081" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1081" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1081" s="3" t="n">
+        <v>314.7587</v>
+      </c>
+      <c r="J1081" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1081" s="3" t="n">
+        <v>314758.7</v>
+      </c>
+      <c r="L1081" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="n">
+        <v>1081</v>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1082" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 12x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1082" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1082" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1082" s="3" t="n">
+        <v>365.0258</v>
+      </c>
+      <c r="J1082" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1082" s="3" t="n">
+        <v>365025.8</v>
+      </c>
+      <c r="L1082" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="n">
+        <v>1082</v>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1083" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 16x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1083" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1083" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1083" s="3" t="n">
+        <v>477.8021</v>
+      </c>
+      <c r="J1083" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1083" s="3" t="n">
+        <v>477802.1</v>
+      </c>
+      <c r="L1083" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="n">
+        <v>1083</v>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1084" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 20x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1084" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1084" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1084" s="3" t="n">
+        <v>590.9489</v>
+      </c>
+      <c r="J1084" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1084" s="3" t="n">
+        <v>590948.9</v>
+      </c>
+      <c r="L1084" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="n">
+        <v>1084</v>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1085" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1085" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl PIMF BLACK 24x2x1,5 mm2 EN 50288-7 500V 70C RAL 9005 Black</t>
+        </is>
+      </c>
+      <c r="G1085" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H1085" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1085" s="3" t="n">
+        <v>698.4758</v>
+      </c>
+      <c r="J1085" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1085" s="3" t="n">
+        <v>698475.8</v>
+      </c>
+      <c r="L1085" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="n">
+        <v>1085</v>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1086" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>LI2Y(St)CH-PF 2x2x24 AWG RS 485 modbus (%65 TC/SNCU orgu kapama), RAL 7001 Gri</t>
+        </is>
+      </c>
+      <c r="G1086" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1086" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1086" s="3" t="n">
+        <v>26.333</v>
+      </c>
+      <c r="J1086" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1086" s="3" t="n">
+        <v>2633.3</v>
+      </c>
+      <c r="L1086" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="n">
+        <v>1086</v>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>ETA Birkablo (marka: BIRTAS KABLO)</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>202402762</t>
+        </is>
+      </c>
+      <c r="D1087" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>TPAO Sirnak Idil Sahasi Pompaj Istasyonu ve Ham Petrol Depolama Tesisi - Kablo Teklifi</t>
+        </is>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>LI-O2YS(St)CY 1x2x18/1AWG PROFIBUS PA, RAL 5015 Mavi</t>
+        </is>
+      </c>
+      <c r="G1087" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1087" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1087" s="3" t="n">
+        <v>41.8983</v>
+      </c>
+      <c r="J1087" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1087" s="3" t="n">
+        <v>4189.83</v>
+      </c>
+      <c r="L1087" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="n">
+        <v>1087</v>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>PROMEK Egitim ve Danismanlik Endustri Malzemeleri Insaat Taahhut Ithalat Ihracat Sanayi Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>TUM24/002</t>
+        </is>
+      </c>
+      <c r="D1088" s="2" t="n">
+        <v>45570</v>
+      </c>
+      <c r="E1088" t="inlineStr">
+        <is>
+          <t>Kardan Mafsalli Deprem Kompansatoru Teklifi</t>
+        </is>
+      </c>
+      <c r="F1088" t="inlineStr">
+        <is>
+          <t>RT7200600-F PN16 Kardan Mafsalli Deprem Kompansatoru Flansli, DN600, L:1370mm, AISI304 korukli, St37-2 govde</t>
+        </is>
+      </c>
+      <c r="G1088" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1088" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1088" s="3" t="n">
+        <v>138146.4</v>
+      </c>
+      <c r="J1088" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1088" s="3" t="n">
+        <v>138146.4</v>
+      </c>
+      <c r="L1088" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="n">
+        <v>1088</v>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>PROMEK Egitim ve Danismanlik Endustri Malzemeleri Insaat Taahhut Ithalat Ihracat Sanayi Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>TUM24/002</t>
+        </is>
+      </c>
+      <c r="D1089" s="2" t="n">
+        <v>45570</v>
+      </c>
+      <c r="E1089" t="inlineStr">
+        <is>
+          <t>Kardan Mafsalli Deprem Kompansatoru Teklifi</t>
+        </is>
+      </c>
+      <c r="F1089" t="inlineStr">
+        <is>
+          <t>RT7200750-F PN16 Kardan Mafsalli Deprem Kompansatoru Flansli, DN750, L:1370mm, AISI304 korukli, St37-2 govde</t>
+        </is>
+      </c>
+      <c r="G1089" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1089" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1089" s="3" t="n">
+        <v>204859.2</v>
+      </c>
+      <c r="J1089" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1089" s="3" t="n">
+        <v>204859.2</v>
+      </c>
+      <c r="L1089" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="n">
+        <v>1089</v>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>RADSAN</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>KR2400000000592</t>
+        </is>
+      </c>
+      <c r="D1090" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1090" t="inlineStr">
+        <is>
+          <t>Topraklama Malzemeleri Teklifi</t>
+        </is>
+      </c>
+      <c r="F1090" t="inlineStr">
+        <is>
+          <t>MH-08.06.D2 35 mm2 Galvaniz Monotron Iletken tel (7,65 mm)</t>
+        </is>
+      </c>
+      <c r="G1090" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1090" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1090" s="3" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="J1090" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1090" s="3" t="n">
+        <v>2550</v>
+      </c>
+      <c r="L1090" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="n">
+        <v>1090</v>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>RADSAN</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>KR2400000000592</t>
+        </is>
+      </c>
+      <c r="D1091" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1091" t="inlineStr">
+        <is>
+          <t>Topraklama Malzemeleri Teklifi</t>
+        </is>
+      </c>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>CG-101.13.D 50 mikron Sicak galvaniz kapli serit, 40x4mm</t>
+        </is>
+      </c>
+      <c r="G1091" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="H1091" t="inlineStr">
+        <is>
+          <t>Kg</t>
+        </is>
+      </c>
+      <c r="I1091" s="3" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="J1091" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1091" s="3" t="n">
+        <v>4901</v>
+      </c>
+      <c r="L1091" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="n">
+        <v>1091</v>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>RADSAN</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>KR2400000000592</t>
+        </is>
+      </c>
+      <c r="D1092" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1092" t="inlineStr">
+        <is>
+          <t>Topraklama Malzemeleri Teklifi</t>
+        </is>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>NYAF-101.05 16 mm2 NYAF Kablo, sari-yesil</t>
+        </is>
+      </c>
+      <c r="G1092" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1092" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1092" s="3" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="J1092" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1092" s="3" t="n">
+        <v>7050</v>
+      </c>
+      <c r="L1092" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="n">
+        <v>1092</v>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>RADSAN</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>KR2400000000592</t>
+        </is>
+      </c>
+      <c r="D1093" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>Topraklama Malzemeleri Teklifi</t>
+        </is>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>NYAF-101.08 50 mm2 NYAF Kablo, sari-yesil</t>
+        </is>
+      </c>
+      <c r="G1093" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1093" t="inlineStr">
+        <is>
+          <t>Mt</t>
+        </is>
+      </c>
+      <c r="I1093" s="3" t="n">
+        <v>218.35</v>
+      </c>
+      <c r="J1093" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1093" s="3" t="n">
+        <v>21835</v>
+      </c>
+      <c r="L1093" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="n">
+        <v>1093</v>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>RADSAN</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>KR2400000000592</t>
+        </is>
+      </c>
+      <c r="D1094" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1094" t="inlineStr">
+        <is>
+          <t>Topraklama Malzemeleri Teklifi</t>
+        </is>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>RIP.101.01 Topraklama Rogari, 50x60x60 cm, Beton</t>
+        </is>
+      </c>
+      <c r="G1094" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1094" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1094" s="3" t="n">
+        <v>2650</v>
+      </c>
+      <c r="J1094" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1094" s="3" t="n">
+        <v>2650</v>
+      </c>
+      <c r="L1094" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="n">
+        <v>1094</v>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>RADSAN</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>KR2400000000592</t>
+        </is>
+      </c>
+      <c r="D1095" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>Topraklama Malzemeleri Teklifi</t>
+        </is>
+      </c>
+      <c r="F1095" t="inlineStr">
+        <is>
+          <t>EBK.200.02 40x5x300 mm Espotansiyel Bara, Izolatorlu, Sicak galvaniz</t>
+        </is>
+      </c>
+      <c r="G1095" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1095" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1095" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="J1095" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1095" s="3" t="n">
+        <v>215</v>
+      </c>
+      <c r="L1095" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="n">
+        <v>1095</v>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>RADSAN</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>KR2400000000592</t>
+        </is>
+      </c>
+      <c r="D1096" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E1096" t="inlineStr">
+        <is>
+          <t>Topraklama Malzemeleri Teklifi</t>
+        </is>
+      </c>
+      <c r="F1096" t="inlineStr">
+        <is>
+          <t>ELT.104.01 25x25cm Statik Bakir Levha 1mm (TR)</t>
+        </is>
+      </c>
+      <c r="G1096" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1096" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1096" s="3" t="n">
+        <v>850</v>
+      </c>
+      <c r="J1096" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1096" s="3" t="n">
+        <v>850</v>
+      </c>
+      <c r="L1096" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="n">
+        <v>1096</v>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>PROMEK Egitim ve Danismanlik Endustri Malzemeleri Insaat Taahhut Ithalat Ihracat Sanayi Ticaret Ltd. Sti.</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>TUM24/003</t>
+        </is>
+      </c>
+      <c r="D1097" s="2" t="n">
+        <v>45582</v>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>Kardan Mafsalli Deprem Kompansatoru Teklifi</t>
+        </is>
+      </c>
+      <c r="F1097" t="inlineStr">
+        <is>
+          <t>RT7200400-F PN16 Kardan Mafsalli Deprem Kompansatoru Flansli, DN400, L:1400mm, Class150, AISI304 korukli, St37-2 govde</t>
+        </is>
+      </c>
+      <c r="G1097" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1097" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1097" s="3" t="n">
+        <v>103860</v>
+      </c>
+      <c r="J1097" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1097" s="3" t="n">
+        <v>103860</v>
+      </c>
+      <c r="L1097" t="inlineStr">
+        <is>
+          <t>1393A_313480kadar.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1033"/>
+  <autoFilter ref="A1:L1097"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ozdoganplast.pdf proformasini listeye ekle (PE Triplex boru)
Ozdoganplast'tan alinan TKF202600001267 nolu teklif (15 kalem PE Triplex
kanal borusu/mansonu/dirsegi) listeye eklendi. Liste artik 82 proforma /
1111 kalem iceriyor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KcsznZgePm4VouW6FRZtG
</commit_message>
<xml_diff>
--- a/PROFORMA_FIYAT_LISTESI.xlsx
+++ b/PROFORMA_FIYAT_LISTESI.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Kalem Detay" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$82</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1097</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3867,8 +3867,52 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>TL (KDV Dahil)</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="n">
+        <v>381207.07</v>
+      </c>
+      <c r="H83" t="n">
+        <v>15</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Ara Toplam/Brüt Toplam (KDV Hariç) 317.672,56 TL + KDV %20 63.534,51 TL = Genel Toplam 381.207,07 TL</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J82"/>
+  <autoFilter ref="A1:J83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3879,7 +3923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1097"/>
+  <dimension ref="A1:L1112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -60700,8 +60744,788 @@
         </is>
       </c>
     </row>
+    <row r="1098">
+      <c r="A1098" t="n">
+        <v>1097</v>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1098" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1098" t="inlineStr">
+        <is>
+          <t>K200KM8 - 200mm PE SN8 Perforeli Triplex Kanal Borusu</t>
+        </is>
+      </c>
+      <c r="G1098" s="4" t="n">
+        <v>644</v>
+      </c>
+      <c r="H1098" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I1098" s="3" t="n">
+        <v>181.24</v>
+      </c>
+      <c r="J1098" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1098" s="3" t="n">
+        <v>116718.56</v>
+      </c>
+      <c r="L1098" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="n">
+        <v>1098</v>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1099" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1099" t="inlineStr">
+        <is>
+          <t>K200M - 200mm PE Triplex Boru Manşon</t>
+        </is>
+      </c>
+      <c r="G1099" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="H1099" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1099" s="3" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="J1099" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1099" s="3" t="n">
+        <v>5566</v>
+      </c>
+      <c r="L1099" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="n">
+        <v>1099</v>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1100" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1100" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1100" t="inlineStr">
+        <is>
+          <t>K200C - 200mm Triplex Muflu Boru Conta</t>
+        </is>
+      </c>
+      <c r="G1100" s="4" t="n">
+        <v>184</v>
+      </c>
+      <c r="H1100" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1100" s="3" t="n">
+        <v>18.77</v>
+      </c>
+      <c r="J1100" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1100" s="3" t="n">
+        <v>3453.68</v>
+      </c>
+      <c r="L1100" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="n">
+        <v>1100</v>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1101" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1101" t="inlineStr">
+        <is>
+          <t>K200KM8 - 200mm PE SN8 Triplex Muflu Boru</t>
+        </is>
+      </c>
+      <c r="G1101" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="H1101" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I1101" s="3" t="n">
+        <v>168.94</v>
+      </c>
+      <c r="J1101" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1101" s="3" t="n">
+        <v>20272.8</v>
+      </c>
+      <c r="L1101" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="n">
+        <v>1101</v>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1102" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1102" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1102" t="inlineStr">
+        <is>
+          <t>K300KM8 - 300mm PE SN8 Perforeli Triplex Kanal Borusu</t>
+        </is>
+      </c>
+      <c r="G1102" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1102" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I1102" s="3" t="n">
+        <v>381.65</v>
+      </c>
+      <c r="J1102" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1102" s="3" t="n">
+        <v>16029.3</v>
+      </c>
+      <c r="L1102" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="n">
+        <v>1102</v>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1103" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1103" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1103" t="inlineStr">
+        <is>
+          <t>K300M - 300mm PE Triplex Boru Manşon</t>
+        </is>
+      </c>
+      <c r="G1103" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1103" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1103" s="3" t="n">
+        <v>140.88</v>
+      </c>
+      <c r="J1103" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1103" s="3" t="n">
+        <v>845.28</v>
+      </c>
+      <c r="L1103" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="n">
+        <v>1103</v>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1104" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1104" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1104" t="inlineStr">
+        <is>
+          <t>K300C - 300mm Triplex Muflu Ek Parça Contası</t>
+        </is>
+      </c>
+      <c r="G1104" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1104" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1104" s="3" t="n">
+        <v>120.47</v>
+      </c>
+      <c r="J1104" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1104" s="3" t="n">
+        <v>1445.64</v>
+      </c>
+      <c r="L1104" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="n">
+        <v>1104</v>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1105" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1105" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1105" t="inlineStr">
+        <is>
+          <t>YDK - 200mm PE Triplex T Çatal 90</t>
+        </is>
+      </c>
+      <c r="G1105" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H1105" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1105" s="3" t="n">
+        <v>262.65</v>
+      </c>
+      <c r="J1105" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1105" s="3" t="n">
+        <v>2889.15</v>
+      </c>
+      <c r="L1105" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="n">
+        <v>1105</v>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1106" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1106" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1106" t="inlineStr">
+        <is>
+          <t>K20045D - 200mm PE Triplex Boru Dirsek (45°)</t>
+        </is>
+      </c>
+      <c r="G1106" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="H1106" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1106" s="3" t="n">
+        <v>119.97</v>
+      </c>
+      <c r="J1106" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1106" s="3" t="n">
+        <v>2999.25</v>
+      </c>
+      <c r="L1106" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="n">
+        <v>1106</v>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1107" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1107" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1107" t="inlineStr">
+        <is>
+          <t>K20090D - 200mm PE Triplex Boru Dirsek (90°)</t>
+        </is>
+      </c>
+      <c r="G1107" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="H1107" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1107" s="3" t="n">
+        <v>154.25</v>
+      </c>
+      <c r="J1107" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1107" s="3" t="n">
+        <v>3393.5</v>
+      </c>
+      <c r="L1107" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="n">
+        <v>1107</v>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1108" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1108" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1108" t="inlineStr">
+        <is>
+          <t>K100KM8 - 100mm PE SN8 Triplex Muflu Boru</t>
+        </is>
+      </c>
+      <c r="G1108" s="4" t="n">
+        <v>174</v>
+      </c>
+      <c r="H1108" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I1108" s="3" t="n">
+        <v>54.89</v>
+      </c>
+      <c r="J1108" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1108" s="3" t="n">
+        <v>9550.860000000001</v>
+      </c>
+      <c r="L1108" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="n">
+        <v>1108</v>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1109" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1109" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1109" t="inlineStr">
+        <is>
+          <t>k100km8 - 100mm PE SN8 Triplex Muflu Boru</t>
+        </is>
+      </c>
+      <c r="G1109" s="4" t="n">
+        <v>660</v>
+      </c>
+      <c r="H1109" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I1109" s="3" t="n">
+        <v>54.89</v>
+      </c>
+      <c r="J1109" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1109" s="3" t="n">
+        <v>36227.4</v>
+      </c>
+      <c r="L1109" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="n">
+        <v>1109</v>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1110" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1110" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1110" t="inlineStr">
+        <is>
+          <t>k100km8 - 100mm PE SN8 Triplex Muflu Boru</t>
+        </is>
+      </c>
+      <c r="G1110" s="4" t="n">
+        <v>702</v>
+      </c>
+      <c r="H1110" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I1110" s="3" t="n">
+        <v>54.89</v>
+      </c>
+      <c r="J1110" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1110" s="3" t="n">
+        <v>38532.78</v>
+      </c>
+      <c r="L1110" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="n">
+        <v>1110</v>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1111" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1111" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1111" t="inlineStr">
+        <is>
+          <t>k100km8 - 100mm PE SN8 Triplex Muflu Boru</t>
+        </is>
+      </c>
+      <c r="G1111" s="4" t="n">
+        <v>924</v>
+      </c>
+      <c r="H1111" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I1111" s="3" t="n">
+        <v>54.89</v>
+      </c>
+      <c r="J1111" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1111" s="3" t="n">
+        <v>50718.36</v>
+      </c>
+      <c r="L1111" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="n">
+        <v>1111</v>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>ÖZDOĞANPLAST PLASTİK VE KİM.MAD.PAZ.SAN.VE TİC.LTD.ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>TKF202600001267</t>
+        </is>
+      </c>
+      <c r="D1112" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1112" t="inlineStr">
+        <is>
+          <t>Genel Malzeme Talebi (PE Triplex Boru/Kanal Sistemi)</t>
+        </is>
+      </c>
+      <c r="F1112" t="inlineStr">
+        <is>
+          <t>k150km8 - 150mm PE SN8 Triplex Muflu Boru</t>
+        </is>
+      </c>
+      <c r="G1112" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="H1112" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="I1112" s="3" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="J1112" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1112" s="3" t="n">
+        <v>9030</v>
+      </c>
+      <c r="L1112" t="inlineStr">
+        <is>
+          <t>ozdoganplast.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1097"/>
+  <autoFilter ref="A1:L1112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
199TPAO_6991374kadar.pdf proformalarini listeye ekle
199TPAO_6991374kadar.pdf icindeki 4 proformadan (Protas Proje/Prosense
exproof ekipman, Seta Celik tank imalati, Patrion pano imalati, Yakan
Aydinlatma direk/armatur) toplam 19 kalem eklendi. Fiyatsiz iki adet
Prosense/R.Stahl terminal box teknik spesifikasyonu (sadece datasheet,
proforma degil) listeye eklenmedi. Liste artik 111 proforma / 1287 kalem
iceriyor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KcsznZgePm4VouW6FRZtG
</commit_message>
<xml_diff>
--- a/PROFORMA_FIYAT_LISTESI.xlsx
+++ b/PROFORMA_FIYAT_LISTESI.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Kalem Detay" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$108</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1269</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1288</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5007,8 +5007,184 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>PROTAŞ PROJE MÜHENDİSLİK (marka: Prosense)</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>VTK03214</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Exproof Ekipman Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="n">
+        <v>1769.45</v>
+      </c>
+      <c r="H109" t="n">
+        <v>6</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Alt Toplam 1.474,54 EUR + KDV 294,91 EUR = Genel Toplam 1.769,45 EUR</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>SETA ÇELİK</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Teklif Konusu: Çelik Tank İmalatı (Rev.1)</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Mehmet İrfan Güler Petrol Üretim İstasyonu - Çelik Tank İmalatı (20.000/7.000/2.000 BBL)</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="n">
+        <v>1005906.27</v>
+      </c>
+      <c r="H110" t="n">
+        <v>6</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>KDV hariç; ağırlıklar yaklaşık, nihai ağırlıklar projelendirme sonrası belli olacak</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>PATRİON İLERİ TEKNOLOJİ SİSTEMLERİ A.Ş.</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>PK100375</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Şırnak ADP + Kompanzasyon Pano İmalatı (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="n">
+        <v>35385.1</v>
+      </c>
+      <c r="H111" t="n">
+        <v>2</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Toplam 29.487,58 EUR + KDV %20 5.897,52 EUR = Genel Toplam 35.385,10 EUR</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>YAKAN AYDINLATMA (Selçuk Yakan)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>003472</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Kamera Direği Malzemeleri (Alıcı: HB Elektrik - Bayram Çolak)</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="n">
+        <v>14875.2</v>
+      </c>
+      <c r="H112" t="n">
+        <v>5</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>İndirimli Toplam (Liste fiyatı üzerinden %45/%0 iskonto) 12.396,00 USD + KDV %20 2.479,20 USD = Toplam Tutar 14.875,20 USD. Not: Prosense/R.Stahl marka iki adet 'Terminal Box Ex e' teknik teklifi (Proposal 33328/33329 Rev.0) bu dosyada fiyatsız (sadece teknik spesifikasyon) olarak yer alıyor, listeye eklenmedi.</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J108"/>
+  <autoFilter ref="A1:J112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5019,7 +5195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1269"/>
+  <dimension ref="A1:L1288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -70782,8 +70958,996 @@
         </is>
       </c>
     </row>
+    <row r="1270">
+      <c r="A1270" t="n">
+        <v>1269</v>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>PROTAŞ PROJE MÜHENDİSLİK (marka: Prosense)</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>VTK03214</t>
+        </is>
+      </c>
+      <c r="D1270" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>Exproof Ekipman Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1270" t="inlineStr">
+        <is>
+          <t>EVFRL.236-NK Ex-proof LED Floresan Aydınlatma Armatürü, 2x45W, 11880 Lümen, Ex-d Zone1/21</t>
+        </is>
+      </c>
+      <c r="G1270" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1270" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1270" s="3" t="n">
+        <v>369.6</v>
+      </c>
+      <c r="J1270" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1270" s="3" t="n">
+        <v>1108.8</v>
+      </c>
+      <c r="L1270" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="n">
+        <v>1270</v>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>PROTAŞ PROJE MÜHENDİSLİK (marka: Prosense)</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>VTK03214</t>
+        </is>
+      </c>
+      <c r="D1271" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>Exproof Ekipman Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1271" t="inlineStr">
+        <is>
+          <t>EFSC.21 Ex-proof Monofaze Elektrik Anahtarı (0-1 Aç/Kapa), 1x20A, 3/4NPT, Zone1/21</t>
+        </is>
+      </c>
+      <c r="G1271" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1271" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1271" s="3" t="n">
+        <v>48.12</v>
+      </c>
+      <c r="J1271" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1271" s="3" t="n">
+        <v>48.12</v>
+      </c>
+      <c r="L1271" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="n">
+        <v>1271</v>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>PROTAŞ PROJE MÜHENDİSLİK (marka: Prosense)</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>VTK03214</t>
+        </is>
+      </c>
+      <c r="D1272" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>Exproof Ekipman Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1272" t="inlineStr">
+        <is>
+          <t>GUFT.26 Ayaklı Ex-proof Bağlantı Buatı, Üç Girişli, 133x133x82mm, IP6X, Ex-d, Zone1/21</t>
+        </is>
+      </c>
+      <c r="G1272" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1272" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1272" s="3" t="n">
+        <v>17.32</v>
+      </c>
+      <c r="J1272" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1272" s="3" t="n">
+        <v>17.32</v>
+      </c>
+      <c r="L1272" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="n">
+        <v>1272</v>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>PROTAŞ PROJE MÜHENDİSLİK (marka: Prosense)</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>VTK03214</t>
+        </is>
+      </c>
+      <c r="D1273" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>Exproof Ekipman Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1273" t="inlineStr">
+        <is>
+          <t>KBA-2M Ex-proof Zırhlı Kablo Rakoru, IP66, M25x1.5, Sıkma Aralığı 12-21mm</t>
+        </is>
+      </c>
+      <c r="G1273" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1273" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1273" s="3" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="J1273" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1273" s="3" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="L1273" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="n">
+        <v>1273</v>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>PROTAŞ PROJE MÜHENDİSLİK (marka: Prosense)</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>VTK03214</t>
+        </is>
+      </c>
+      <c r="D1274" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>Exproof Ekipman Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>KBA-5M Ex-proof Zırhlı Kablo Rakoru, IP66, M50x1.5, Sıkma Aralığı 36-52mm</t>
+        </is>
+      </c>
+      <c r="G1274" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1274" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1274" s="3" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="J1274" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1274" s="3" t="n">
+        <v>184.8</v>
+      </c>
+      <c r="L1274" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="n">
+        <v>1274</v>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>PROTAŞ PROJE MÜHENDİSLİK (marka: Prosense)</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>VTK03214</t>
+        </is>
+      </c>
+      <c r="D1275" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>Exproof Ekipman Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>KBA-1M Ex-proof Zırhlı Kablo Rakoru, IP66, M20x1.5, Sıkma Aralığı 8.5-16mm</t>
+        </is>
+      </c>
+      <c r="G1275" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H1275" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1275" s="3" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="J1275" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1275" s="3" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="L1275" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="n">
+        <v>1275</v>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>SETA ÇELİK</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Teklif Konusu: Çelik Tank İmalatı (Rev.1)</t>
+        </is>
+      </c>
+      <c r="D1276" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>Mehmet İrfan Güler Petrol Üretim İstasyonu - Çelik Tank İmalatı (20.000/7.000/2.000 BBL)</t>
+        </is>
+      </c>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>20.000 BBL Çelik Tank İmalatı (Ø19000mm H12021mm, S275JR, Dikey Silindirik Atmosferik, Konik Çatı) - İmalat</t>
+        </is>
+      </c>
+      <c r="G1276" s="4" t="n">
+        <v>121587.9</v>
+      </c>
+      <c r="H1276" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="I1276" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1276" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1276" s="3" t="n">
+        <v>243175.8</v>
+      </c>
+      <c r="L1276" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="n">
+        <v>1276</v>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>SETA ÇELİK</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>Teklif Konusu: Çelik Tank İmalatı (Rev.1)</t>
+        </is>
+      </c>
+      <c r="D1277" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>Mehmet İrfan Güler Petrol Üretim İstasyonu - Çelik Tank İmalatı (20.000/7.000/2.000 BBL)</t>
+        </is>
+      </c>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>20.000 BBL Çelik Tank Montajı</t>
+        </is>
+      </c>
+      <c r="G1277" s="4" t="n">
+        <v>121587.9</v>
+      </c>
+      <c r="H1277" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="I1277" s="3" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J1277" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1277" s="3" t="n">
+        <v>449875.23</v>
+      </c>
+      <c r="L1277" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="n">
+        <v>1277</v>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>SETA ÇELİK</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Teklif Konusu: Çelik Tank İmalatı (Rev.1)</t>
+        </is>
+      </c>
+      <c r="D1278" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>Mehmet İrfan Güler Petrol Üretim İstasyonu - Çelik Tank İmalatı (20.000/7.000/2.000 BBL)</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>7.000 BBL Çelik Tank İmalatı (Ø12730mm H8920mm, S275JR, Dikey Silindirik Atmosferik, Konik Çatı) - İmalat</t>
+        </is>
+      </c>
+      <c r="G1278" s="4" t="n">
+        <v>37714.1</v>
+      </c>
+      <c r="H1278" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="I1278" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1278" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1278" s="3" t="n">
+        <v>75428.2</v>
+      </c>
+      <c r="L1278" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="n">
+        <v>1278</v>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>SETA ÇELİK</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Teklif Konusu: Çelik Tank İmalatı (Rev.1)</t>
+        </is>
+      </c>
+      <c r="D1279" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>Mehmet İrfan Güler Petrol Üretim İstasyonu - Çelik Tank İmalatı (20.000/7.000/2.000 BBL)</t>
+        </is>
+      </c>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>7.000 BBL Çelik Tank Montajı</t>
+        </is>
+      </c>
+      <c r="G1279" s="4" t="n">
+        <v>37714.1</v>
+      </c>
+      <c r="H1279" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="I1279" s="3" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J1279" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1279" s="3" t="n">
+        <v>139542.17</v>
+      </c>
+      <c r="L1279" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="n">
+        <v>1279</v>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>SETA ÇELİK</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>Teklif Konusu: Çelik Tank İmalatı (Rev.1)</t>
+        </is>
+      </c>
+      <c r="D1280" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>Mehmet İrfan Güler Petrol Üretim İstasyonu - Çelik Tank İmalatı (20.000/7.000/2.000 BBL)</t>
+        </is>
+      </c>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>2.000 BBL Çelik Tank İmalatı (Ø7000mm H9000mm, ST52, Dikey Silindirik Atmosferik, Konik Çatı) - İmalat</t>
+        </is>
+      </c>
+      <c r="G1280" s="4" t="n">
+        <v>16046.7</v>
+      </c>
+      <c r="H1280" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="I1280" s="3" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J1280" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1280" s="3" t="n">
+        <v>36907.41</v>
+      </c>
+      <c r="L1280" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="n">
+        <v>1280</v>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>SETA ÇELİK</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>Teklif Konusu: Çelik Tank İmalatı (Rev.1)</t>
+        </is>
+      </c>
+      <c r="D1281" s="2" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>Mehmet İrfan Güler Petrol Üretim İstasyonu - Çelik Tank İmalatı (20.000/7.000/2.000 BBL)</t>
+        </is>
+      </c>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>2.000 BBL Çelik Tank Montajı</t>
+        </is>
+      </c>
+      <c r="G1281" s="4" t="n">
+        <v>16046.7</v>
+      </c>
+      <c r="H1281" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="I1281" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="J1281" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1281" s="3" t="n">
+        <v>60977.46</v>
+      </c>
+      <c r="L1281" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="n">
+        <v>1281</v>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>PATRİON İLERİ TEKNOLOJİ SİSTEMLERİ A.Ş.</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>PK100375</t>
+        </is>
+      </c>
+      <c r="D1282" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>Şırnak ADP + Kompanzasyon Pano İmalatı (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>ŞIRNAK ADP Panosu, EAE ES IP55 FORM4B 2000+100x(500+500+400+600+300+600+400)x600mm</t>
+        </is>
+      </c>
+      <c r="G1282" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1282" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1282" s="3" t="n">
+        <v>25779.79</v>
+      </c>
+      <c r="J1282" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1282" s="3" t="n">
+        <v>25779.79</v>
+      </c>
+      <c r="L1282" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="n">
+        <v>1282</v>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>PATRİON İLERİ TEKNOLOJİ SİSTEMLERİ A.Ş.</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>PK100375</t>
+        </is>
+      </c>
+      <c r="D1283" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>Şırnak ADP + Kompanzasyon Pano İmalatı (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>ŞIRNAK KOMPANZASYON Panosu, EAE ES IP55 FORM2B 2000+100x(600)x600mm</t>
+        </is>
+      </c>
+      <c r="G1283" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1283" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1283" s="3" t="n">
+        <v>3707.79</v>
+      </c>
+      <c r="J1283" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1283" s="3" t="n">
+        <v>3707.79</v>
+      </c>
+      <c r="L1283" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="n">
+        <v>1283</v>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>YAKAN AYDINLATMA (Selçuk Yakan)</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>003472</t>
+        </is>
+      </c>
+      <c r="D1284" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Kamera Direği Malzemeleri (Alıcı: HB Elektrik - Bayram Çolak)</t>
+        </is>
+      </c>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>K-95100 Poligon Direk Tek Konsol Galvanizli 10M</t>
+        </is>
+      </c>
+      <c r="G1284" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1284" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1284" s="3" t="n">
+        <v>338.25</v>
+      </c>
+      <c r="J1284" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1284" s="3" t="n">
+        <v>6088.5</v>
+      </c>
+      <c r="L1284" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="n">
+        <v>1284</v>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>YAKAN AYDINLATMA (Selçuk Yakan)</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>003472</t>
+        </is>
+      </c>
+      <c r="D1285" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Kamera Direği Malzemeleri (Alıcı: HB Elektrik - Bayram Çolak)</t>
+        </is>
+      </c>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>225104 ZEYA 100W 4000K LED Armatür IP66 (ZL-ST22G-100W)</t>
+        </is>
+      </c>
+      <c r="G1285" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1285" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1285" s="3" t="n">
+        <v>26.95</v>
+      </c>
+      <c r="J1285" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1285" s="3" t="n">
+        <v>485.1</v>
+      </c>
+      <c r="L1285" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="n">
+        <v>1285</v>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>YAKAN AYDINLATMA (Selçuk Yakan)</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>003472</t>
+        </is>
+      </c>
+      <c r="D1286" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Kamera Direği Malzemeleri (Alıcı: HB Elektrik - Bayram Çolak)</t>
+        </is>
+      </c>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>99005 Kamera Direği Çelik Boru 5 Metre</t>
+        </is>
+      </c>
+      <c r="G1286" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1286" s="3" t="n">
+        <v>91.28</v>
+      </c>
+      <c r="J1286" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1286" s="3" t="n">
+        <v>365.13</v>
+      </c>
+      <c r="L1286" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="n">
+        <v>1286</v>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>YAKAN AYDINLATMA (Selçuk Yakan)</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>003472</t>
+        </is>
+      </c>
+      <c r="D1287" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Kamera Direği Malzemeleri (Alıcı: HB Elektrik - Bayram Çolak)</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>98880 Lazer Kamera Makaralı Konsol Tekli</t>
+        </is>
+      </c>
+      <c r="G1287" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1287" s="3" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="J1287" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1287" s="3" t="n">
+        <v>57.26</v>
+      </c>
+      <c r="L1287" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="n">
+        <v>1287</v>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>YAKAN AYDINLATMA (Selçuk Yakan)</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>003472</t>
+        </is>
+      </c>
+      <c r="D1288" s="2" t="n">
+        <v>46162</v>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Kamera Direği Malzemeleri (Alıcı: HB Elektrik - Bayram Çolak)</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>S01680-1 Galvanizleme (Elektro Galvanizleme)</t>
+        </is>
+      </c>
+      <c r="G1288" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1288" s="3" t="n">
+        <v>1350</v>
+      </c>
+      <c r="J1288" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1288" s="3" t="n">
+        <v>5400</v>
+      </c>
+      <c r="L1288" t="inlineStr">
+        <is>
+          <t>199TPAO_6991374kadar.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1269"/>
+  <autoFilter ref="A1:L1288"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
199TPAO_13741768kadar.pdf proformalarini listeye ekle
Borusan Makina (Caterpillar dizel jenerator, DE660E0/DE660GC alternatifli)
ve Marmara Direk Aydinlatma (poligon direk) teklifleri eklendi. Liste
artik 113 proforma / 1292 kalem iceriyor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KcsznZgePm4VouW6FRZtG
</commit_message>
<xml_diff>
--- a/PROFORMA_FIYAT_LISTESI.xlsx
+++ b/PROFORMA_FIYAT_LISTESI.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Kalem Detay" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1288</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1293</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J112"/>
+  <dimension ref="A1:J114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5183,8 +5183,96 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>BORUSAN MAKİNA VE GÜÇ SİSTEMLERİ SANAYİ VE TİCARET A.Ş.</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Ref yok (09.06.2026 Teklif Mektubu)</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Şırnak MİG Petrol Depolama Tesisi - Dizel Jeneratör Seti</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="n">
+        <v>115000</v>
+      </c>
+      <c r="H113" t="n">
+        <v>2</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>KDV Hariç. ALTERNATİF (veya): Aynı teklifte CATERPILLAR DE660GC 660KVA Standby (Prime çalışmaya uygun değil) modeli 105.000 EUR KDV Hariç olarak da sunulmuş - iki model birbirinin alternatifi, toplama dahil değil, sadece biri seçilecek. Socomec ATS panosu opsiyoneldir, her iki model için de geçerlidir. Ödeme %30 avans + %70 sevkiyat öncesi.</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>199TPAO_13741768kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>MARMARA DİREK AYDINLATMA SAN. TİC. LTD. ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>1540</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Paratoner/Kamera Direği Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="n">
+        <v>367920</v>
+      </c>
+      <c r="H114" t="n">
+        <v>3</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Toplam 306.600,00 TL + KDV %20 61.320,00 TL = Genel Toplam 367.920,00 TL. Teslim Yeri İstanbul Fabrika, teslim süresi 4-6 hafta.</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>199TPAO_13741768kadar.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J112"/>
+  <autoFilter ref="A1:J114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5195,7 +5283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1288"/>
+  <dimension ref="A1:L1293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -71946,8 +72034,268 @@
         </is>
       </c>
     </row>
+    <row r="1289">
+      <c r="A1289" t="n">
+        <v>1288</v>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>BORUSAN MAKİNA VE GÜÇ SİSTEMLERİ SANAYİ VE TİCARET A.Ş.</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>Ref yok (09.06.2026 Teklif Mektubu)</t>
+        </is>
+      </c>
+      <c r="D1289" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>Şırnak MİG Petrol Depolama Tesisi - Dizel Jeneratör Seti</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>CATERPILLAR DE660E0 660KVA Standby/600KVA Prime 400V 50Hz 0.8PF 1500RPM Dizel Jeneratör Seti (kontrol paneli, redresör, akü grubu, susturucu, giydirme kabin, alternatör koruma şalteri, nakliye ve devreye alma dahil)</t>
+        </is>
+      </c>
+      <c r="G1289" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1289" s="3" t="n">
+        <v>115000</v>
+      </c>
+      <c r="J1289" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1289" s="3" t="n">
+        <v>115000</v>
+      </c>
+      <c r="L1289" t="inlineStr">
+        <is>
+          <t>199TPAO_13741768kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="n">
+        <v>1289</v>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>BORUSAN MAKİNA VE GÜÇ SİSTEMLERİ SANAYİ VE TİCARET A.Ş.</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Ref yok (09.06.2026 Teklif Mektubu)</t>
+        </is>
+      </c>
+      <c r="D1290" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>Şırnak MİG Petrol Depolama Tesisi - Dizel Jeneratör Seti</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>Opsiyonel: Socomec Otomatik Transfer Panosu</t>
+        </is>
+      </c>
+      <c r="G1290" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1290" s="3" t="n">
+        <v>5250</v>
+      </c>
+      <c r="J1290" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="K1290" s="3" t="n">
+        <v>5250</v>
+      </c>
+      <c r="L1290" t="inlineStr">
+        <is>
+          <t>199TPAO_13741768kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="n">
+        <v>1290</v>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>MARMARA DİREK AYDINLATMA SAN. TİC. LTD. ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>1540</t>
+        </is>
+      </c>
+      <c r="D1291" s="2" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Paratoner/Kamera Direği Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>10 MT Galvaniz Poligon Aydınlatma Direği Tek Konsol + Tek Kamera Konsollu</t>
+        </is>
+      </c>
+      <c r="G1291" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1291" s="3" t="n">
+        <v>10950</v>
+      </c>
+      <c r="J1291" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1291" s="3" t="n">
+        <v>197100</v>
+      </c>
+      <c r="L1291" t="inlineStr">
+        <is>
+          <t>199TPAO_13741768kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="n">
+        <v>1291</v>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>MARMARA DİREK AYDINLATMA SAN. TİC. LTD. ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>1540</t>
+        </is>
+      </c>
+      <c r="D1292" s="2" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Paratoner/Kamera Direği Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>19 MT Galvaniz Poligon Paratoner Direği</t>
+        </is>
+      </c>
+      <c r="G1292" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1292" s="3" t="n">
+        <v>45750</v>
+      </c>
+      <c r="J1292" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1292" s="3" t="n">
+        <v>91500</v>
+      </c>
+      <c r="L1292" t="inlineStr">
+        <is>
+          <t>199TPAO_13741768kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="n">
+        <v>1292</v>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>MARMARA DİREK AYDINLATMA SAN. TİC. LTD. ŞTİ.</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>1540</t>
+        </is>
+      </c>
+      <c r="D1293" s="2" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>Aydınlatma/Paratoner/Kamera Direği Talebi (Firma: HB Elektrik)</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>5 MT Galvaniz Poligon Kamera Direği</t>
+        </is>
+      </c>
+      <c r="G1293" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="I1293" s="3" t="n">
+        <v>4500</v>
+      </c>
+      <c r="J1293" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="K1293" s="3" t="n">
+        <v>18000</v>
+      </c>
+      <c r="L1293" t="inlineStr">
+        <is>
+          <t>199TPAO_13741768kadar.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1288"/>
+  <autoFilter ref="A1:L1293"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1393A_10992064kadar.pdf: 2M Kablo proformasini ekle
Bu dosyanin buyuk kismi daha once islenmis METRANS pompa teklifinin
devami (~3400 satir, bilinen kopya, atlandi) ve Seba Celik Boru'nun genel
fiyat katalogu (musteri/miktar/toplam icermeyen rate card, atlandi) idi.
Sadece 1 yeni musteriye ozel proforma bulundu: 2M Kablo (12 kalem, 5.052
USD). Liste artik 114 proforma / 1304 kalem iceriyor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014KcsznZgePm4VouW6FRZtG
</commit_message>
<xml_diff>
--- a/PROFORMA_FIYAT_LISTESI.xlsx
+++ b/PROFORMA_FIYAT_LISTESI.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Kalem Detay" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$114</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1293</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proforma Özeti'!$A$1:$J$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kalem Detay'!$A$1:$L$1305</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J114"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5271,8 +5271,47 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="n">
+        <v>5052</v>
+      </c>
+      <c r="H115" t="n">
+        <v>12</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Not: TÜRKİYE PETROLLERİ (TPAO); Teklif Formu, Hazırlayan Hasan Ertürk; TOPLAM MİKTAR 1.200,00 m</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J114"/>
+  <autoFilter ref="A1:J115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5283,7 +5322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1293"/>
+  <dimension ref="A1:L1305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -72294,8 +72333,572 @@
         </is>
       </c>
     </row>
+    <row r="1294">
+      <c r="A1294" t="n">
+        <v>1293</v>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1294" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl 1x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1294" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1294" s="3" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="J1294" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1294" s="3" t="n">
+        <v>148</v>
+      </c>
+      <c r="L1294" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="n">
+        <v>1294</v>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1295" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl-PiMF 2x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1295" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1295" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J1295" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1295" s="3" t="n">
+        <v>260</v>
+      </c>
+      <c r="L1295" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="n">
+        <v>1295</v>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1296" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl-PiMF 4x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1296" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1296" s="3" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="J1296" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1296" s="3" t="n">
+        <v>395</v>
+      </c>
+      <c r="L1296" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="n">
+        <v>1296</v>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1297" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl-PiMF 5x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1297" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1297" s="3" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="J1297" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1297" s="3" t="n">
+        <v>477</v>
+      </c>
+      <c r="L1297" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="n">
+        <v>1297</v>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1298" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl-PiMF 6x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1298" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1298" s="3" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="J1298" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1298" s="3" t="n">
+        <v>593</v>
+      </c>
+      <c r="L1298" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="n">
+        <v>1298</v>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1299" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl-PiMF 8x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1299" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1299" s="3" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="J1299" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1299" s="3" t="n">
+        <v>733</v>
+      </c>
+      <c r="L1299" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="n">
+        <v>1299</v>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1300" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl-PiMF 10x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1300" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1300" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="J1300" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1300" s="3" t="n">
+        <v>900</v>
+      </c>
+      <c r="L1300" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="n">
+        <v>1300</v>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1301" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>RE-2X(St)YSWAY-fl-PiMF 12x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1301" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1301" s="3" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="J1301" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1301" s="3" t="n">
+        <v>1049</v>
+      </c>
+      <c r="L1301" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="n">
+        <v>1301</v>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1302" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>LI2Y(St)CH 2x2x0.22 mm2 RS-485 (RAL7001-Grey)</t>
+        </is>
+      </c>
+      <c r="G1302" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1302" s="3" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J1302" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1302" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="L1302" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="n">
+        <v>1302</v>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1303" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>RE-2Y(St)YSWAY-fl 1x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1303" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1303" s="3" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J1303" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1303" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="L1303" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="n">
+        <v>1303</v>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1304" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>RE-2Y(St)YSWAY-fl 2x2x1.5 mm2 500V (RAL5015-Blue)</t>
+        </is>
+      </c>
+      <c r="G1304" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1304" s="3" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="J1304" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1304" s="3" t="n">
+        <v>218</v>
+      </c>
+      <c r="L1304" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="n">
+        <v>1304</v>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>2M KABLO</t>
+        </is>
+      </c>
+      <c r="D1305" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>TÜMAŞ Türk Müh. - TPAO İdil Sahası kablo talebi</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>YSLYCY-OZ 2x1.5 mm2 (RAL7001-Grey)</t>
+        </is>
+      </c>
+      <c r="G1305" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I1305" s="3" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J1305" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K1305" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="L1305" t="inlineStr">
+        <is>
+          <t>1393A_10992064kadar.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L1293"/>
+  <autoFilter ref="A1:L1305"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>